<commit_message>
- Updated employees_data.json and employees_data.xlsx with new employee records and ensured proper formatting.
</commit_message>
<xml_diff>
--- a/Python_Libraries/Pandas/employees_data.xlsx
+++ b/Python_Libraries/Pandas/employees_data.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -46,8 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -506,10 +510,8 @@
       <c r="H2" t="n">
         <v>2</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>2022-01-15</t>
-        </is>
+      <c r="I2" s="1" t="n">
+        <v>44576</v>
       </c>
       <c r="J2" t="n">
         <v>85</v>
@@ -553,10 +555,8 @@
       <c r="H3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>2024-03-10</t>
-        </is>
+      <c r="I3" s="1" t="n">
+        <v>45361</v>
       </c>
       <c r="J3" t="n">
         <v>90</v>
@@ -600,10 +600,8 @@
       <c r="H4" t="n">
         <v>4</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2021-06-20</t>
-        </is>
+      <c r="I4" s="1" t="n">
+        <v>44367</v>
       </c>
       <c r="J4" t="n">
         <v>78</v>
@@ -647,10 +645,8 @@
       <c r="H5" t="n">
         <v>5</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2020-09-01</t>
-        </is>
+      <c r="I5" s="1" t="n">
+        <v>44075</v>
       </c>
       <c r="J5" t="n">
         <v>82</v>
@@ -694,10 +690,8 @@
       <c r="H6" t="n">
         <v>3</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2022-11-12</t>
-        </is>
+      <c r="I6" s="1" t="n">
+        <v>44877</v>
       </c>
       <c r="J6" t="n">
         <v>88</v>
@@ -741,10 +735,8 @@
       <c r="H7" t="n">
         <v>2</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2023-02-05</t>
-        </is>
+      <c r="I7" s="1" t="n">
+        <v>44962</v>
       </c>
       <c r="J7" t="n">
         <v>75</v>
@@ -788,10 +780,8 @@
       <c r="H8" t="n">
         <v>8</v>
       </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>2018-07-18</t>
-        </is>
+      <c r="I8" s="1" t="n">
+        <v>43299</v>
       </c>
       <c r="J8" t="n">
         <v>91</v>
@@ -835,10 +825,8 @@
       <c r="H9" t="n">
         <v>4</v>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>2021-12-01</t>
-        </is>
+      <c r="I9" s="1" t="n">
+        <v>44531</v>
       </c>
       <c r="J9" t="n">
         <v>86</v>
@@ -882,10 +870,8 @@
       <c r="H10" t="n">
         <v>5</v>
       </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>2020-05-22</t>
-        </is>
+      <c r="I10" s="1" t="n">
+        <v>43973</v>
       </c>
       <c r="J10" t="n">
         <v>80</v>
@@ -929,10 +915,8 @@
       <c r="H11" t="n">
         <v>3</v>
       </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>2022-08-30</t>
-        </is>
+      <c r="I11" s="1" t="n">
+        <v>44803</v>
       </c>
       <c r="J11" t="n">
         <v>84</v>
@@ -976,10 +960,8 @@
       <c r="H12" t="n">
         <v>7</v>
       </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>2019-04-14</t>
-        </is>
+      <c r="I12" s="1" t="n">
+        <v>43569</v>
       </c>
       <c r="J12" t="n">
         <v>89</v>
@@ -1023,10 +1005,8 @@
       <c r="H13" t="n">
         <v>1</v>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>2024-01-10</t>
-        </is>
+      <c r="I13" s="1" t="n">
+        <v>45301</v>
       </c>
       <c r="J13" t="n">
         <v>92</v>
@@ -1070,10 +1050,8 @@
       <c r="H14" t="n">
         <v>2</v>
       </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>2023-06-25</t>
-        </is>
+      <c r="I14" s="1" t="n">
+        <v>45102</v>
       </c>
       <c r="J14" t="n">
         <v>76</v>
@@ -1117,10 +1095,8 @@
       <c r="H15" t="n">
         <v>10</v>
       </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>2016-03-19</t>
-        </is>
+      <c r="I15" s="1" t="n">
+        <v>42448</v>
       </c>
       <c r="J15" t="n">
         <v>95</v>
@@ -1164,10 +1140,8 @@
       <c r="H16" t="n">
         <v>2</v>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>2023-09-08</t>
-        </is>
+      <c r="I16" s="1" t="n">
+        <v>45177</v>
       </c>
       <c r="J16" t="n">
         <v>81</v>
@@ -1211,10 +1185,8 @@
       <c r="H17" t="n">
         <v>4</v>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>2021-10-11</t>
-        </is>
+      <c r="I17" s="1" t="n">
+        <v>44480</v>
       </c>
       <c r="J17" t="n">
         <v>87</v>
@@ -1258,10 +1230,8 @@
       <c r="H18" t="n">
         <v>6</v>
       </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>2020-01-27</t>
-        </is>
+      <c r="I18" s="1" t="n">
+        <v>43857</v>
       </c>
       <c r="J18" t="n">
         <v>83</v>
@@ -1305,10 +1275,8 @@
       <c r="H19" t="n">
         <v>3</v>
       </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>2022-04-09</t>
-        </is>
+      <c r="I19" s="1" t="n">
+        <v>44660</v>
       </c>
       <c r="J19" t="n">
         <v>90</v>
@@ -1352,10 +1320,8 @@
       <c r="H20" t="n">
         <v>1</v>
       </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>2024-05-01</t>
-        </is>
+      <c r="I20" s="1" t="n">
+        <v>45413</v>
       </c>
       <c r="J20" t="n">
         <v>74</v>
@@ -1399,10 +1365,8 @@
       <c r="H21" t="n">
         <v>5</v>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>2021-07-15</t>
-        </is>
+      <c r="I21" s="1" t="n">
+        <v>44392</v>
       </c>
       <c r="J21" t="n">
         <v>85</v>
@@ -1446,10 +1410,8 @@
       <c r="H22" t="n">
         <v>6</v>
       </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>2020-11-23</t>
-        </is>
+      <c r="I22" s="1" t="n">
+        <v>44158</v>
       </c>
       <c r="J22" t="n">
         <v>88</v>
@@ -1493,10 +1455,8 @@
       <c r="H23" t="n">
         <v>2</v>
       </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>2023-01-12</t>
-        </is>
+      <c r="I23" s="1" t="n">
+        <v>44938</v>
       </c>
       <c r="J23" t="n">
         <v>86</v>
@@ -1540,10 +1500,8 @@
       <c r="H24" t="n">
         <v>4</v>
       </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>2021-09-18</t>
-        </is>
+      <c r="I24" s="1" t="n">
+        <v>44457</v>
       </c>
       <c r="J24" t="n">
         <v>79</v>
@@ -1587,10 +1545,8 @@
       <c r="H25" t="n">
         <v>2</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>2023-04-20</t>
-        </is>
+      <c r="I25" s="1" t="n">
+        <v>45036</v>
       </c>
       <c r="J25" t="n">
         <v>77</v>
@@ -1634,10 +1590,8 @@
       <c r="H26" t="n">
         <v>9</v>
       </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>2017-12-10</t>
-        </is>
+      <c r="I26" s="1" t="n">
+        <v>43079</v>
       </c>
       <c r="J26" t="n">
         <v>93</v>
@@ -1681,10 +1635,8 @@
       <c r="H27" t="n">
         <v>3</v>
       </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>2022-06-05</t>
-        </is>
+      <c r="I27" s="1" t="n">
+        <v>44717</v>
       </c>
       <c r="J27" t="n">
         <v>82</v>
@@ -1728,10 +1680,8 @@
       <c r="H28" t="n">
         <v>5</v>
       </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>2020-08-28</t>
-        </is>
+      <c r="I28" s="1" t="n">
+        <v>44071</v>
       </c>
       <c r="J28" t="n">
         <v>84</v>
@@ -1775,10 +1725,8 @@
       <c r="H29" t="n">
         <v>4</v>
       </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>2021-03-17</t>
-        </is>
+      <c r="I29" s="1" t="n">
+        <v>44272</v>
       </c>
       <c r="J29" t="n">
         <v>91</v>
@@ -1822,10 +1770,8 @@
       <c r="H30" t="n">
         <v>3</v>
       </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>2022-10-25</t>
-        </is>
+      <c r="I30" s="1" t="n">
+        <v>44859</v>
       </c>
       <c r="J30" t="n">
         <v>78</v>
@@ -1869,10 +1815,8 @@
       <c r="H31" t="n">
         <v>2</v>
       </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>2023-11-02</t>
-        </is>
+      <c r="I31" s="1" t="n">
+        <v>45232</v>
       </c>
       <c r="J31" t="n">
         <v>80</v>

</xml_diff>